<commit_message>
- Wert und Footprint der LED Vorwiderstaende angepasst
</commit_message>
<xml_diff>
--- a/BOM/20211102 BOM TeKaDe Baseboard.xlsx
+++ b/BOM/20211102 BOM TeKaDe Baseboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IngBuero\Projekte_Kunden\2021_TeKaDeRevival\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036C4194-924B-48BE-A425-1248C7E7AA71}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9756184-5EF5-4245-88E4-CD3D31CBEFCF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11960" xr2:uid="{261E8F2A-9F01-4E4B-AED6-14B6866C8B8C}"/>
   </bookViews>
@@ -997,9 +997,6 @@
     <t>Ferrit/470R/1A/0,2R</t>
   </si>
   <si>
-    <t>392R/1%</t>
-  </si>
-  <si>
     <t>10k/1%</t>
   </si>
   <si>
@@ -1379,6 +1376,9 @@
   </si>
   <si>
     <t>Pinheader 1x02 P2,54</t>
+  </si>
+  <si>
+    <t>150R/1%</t>
   </si>
 </sst>
 </file>
@@ -2358,13 +2358,13 @@
         <v>4</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>323</v>
+        <v>450</v>
       </c>
       <c r="D21" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G21" s="9">
-        <v>805</v>
+        <v>603</v>
       </c>
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
@@ -2374,7 +2374,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D22" t="s">
         <v>23</v>
@@ -2390,10 +2390,10 @@
         <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D23" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G23" s="9">
         <v>402</v>
@@ -2406,10 +2406,10 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D24" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G24" s="9">
         <v>402</v>
@@ -2422,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D25" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G25" s="9">
         <v>402</v>
@@ -2438,10 +2438,10 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D26" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G26" s="9">
         <v>402</v>
@@ -2454,10 +2454,10 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D27" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G27" s="9">
         <v>402</v>
@@ -2470,10 +2470,10 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D28" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G28" s="9">
         <v>603</v>
@@ -2486,10 +2486,10 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D29" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="G29" s="9">
         <v>402</v>
@@ -2502,10 +2502,10 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D30" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G30" s="9">
         <v>402</v>
@@ -2518,10 +2518,10 @@
         <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D31" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G31" s="9">
         <v>402</v>
@@ -2534,10 +2534,10 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D32" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G32" s="9">
         <v>402</v>
@@ -2550,10 +2550,10 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D33" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G33" s="9">
         <v>603</v>
@@ -2569,7 +2569,7 @@
         <v>63</v>
       </c>
       <c r="D34" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G34" s="9">
         <v>603</v>
@@ -2582,10 +2582,10 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D35" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G35" s="9">
         <v>402</v>
@@ -2598,10 +2598,10 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D36" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G36" s="9">
         <v>402</v>
@@ -2614,10 +2614,10 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D37" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G37" s="9">
         <v>402</v>
@@ -2630,10 +2630,10 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D38" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G38" s="9">
         <v>402</v>
@@ -2649,7 +2649,7 @@
         <v>298</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G39" s="14">
         <v>402</v>
@@ -2666,7 +2666,7 @@
         <v>298</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G40" s="2">
         <v>603</v>
@@ -2680,10 +2680,10 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D41" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G41" s="9">
         <v>603</v>
@@ -2819,22 +2819,22 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="D47" t="s">
         <v>55</v>
       </c>
       <c r="E47" t="s">
+        <v>406</v>
+      </c>
+      <c r="F47" t="s">
+        <v>405</v>
+      </c>
+      <c r="G47" t="s">
+        <v>354</v>
+      </c>
+      <c r="J47" t="s">
         <v>407</v>
-      </c>
-      <c r="F47" t="s">
-        <v>406</v>
-      </c>
-      <c r="G47" t="s">
-        <v>355</v>
-      </c>
-      <c r="J47" t="s">
-        <v>408</v>
       </c>
       <c r="K47" s="17">
         <v>630</v>
@@ -2854,7 +2854,7 @@
         <v>267</v>
       </c>
       <c r="D48" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E48" s="12" t="s">
         <v>88</v>
@@ -2887,10 +2887,10 @@
         <v>1</v>
       </c>
       <c r="C49" s="38" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D49" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>96</v>
@@ -2922,10 +2922,10 @@
         <v>1</v>
       </c>
       <c r="C50" s="38" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D50" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E50" s="9" t="s">
         <v>96</v>
@@ -2957,10 +2957,10 @@
         <v>1</v>
       </c>
       <c r="C51" s="38" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D51" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>96</v>
@@ -2998,7 +2998,7 @@
         <v>251</v>
       </c>
       <c r="D52" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E52" s="12" t="s">
         <v>246</v>
@@ -3032,7 +3032,7 @@
         <v>247</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E53" s="14" t="s">
         <v>246</v>
@@ -3045,7 +3045,7 @@
         <v>250</v>
       </c>
       <c r="K53" s="29" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="L53" s="34">
         <v>1.25</v>
@@ -3067,7 +3067,7 @@
         <v>262</v>
       </c>
       <c r="D54" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E54" s="9" t="s">
         <v>96</v>
@@ -3100,7 +3100,7 @@
         <v>263</v>
       </c>
       <c r="D55" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>96</v>
@@ -3133,7 +3133,7 @@
         <v>253</v>
       </c>
       <c r="D56" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E56" s="9" t="s">
         <v>252</v>
@@ -3163,22 +3163,22 @@
         <v>1</v>
       </c>
       <c r="C57" s="38" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D57" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G57" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J57" s="9" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K57" s="18">
         <v>44529</v>
@@ -3195,22 +3195,22 @@
         <v>2</v>
       </c>
       <c r="C58" s="38" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D58" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E58" s="9" t="s">
         <v>96</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G58" t="s">
         <v>219</v>
       </c>
       <c r="J58" s="9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K58" s="41">
         <v>110</v>
@@ -3227,23 +3227,23 @@
         <v>0</v>
       </c>
       <c r="C59" s="39" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E59" s="14" t="s">
         <v>96</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>219</v>
       </c>
       <c r="I59" s="25"/>
       <c r="J59" s="14" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="K59" s="23">
         <v>44809</v>
@@ -3260,22 +3260,22 @@
         <v>1</v>
       </c>
       <c r="C60" s="38" t="s">
+        <v>415</v>
+      </c>
+      <c r="D60" t="s">
+        <v>387</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="G60" t="s">
+        <v>356</v>
+      </c>
+      <c r="J60" s="9" t="s">
         <v>416</v>
-      </c>
-      <c r="D60" t="s">
-        <v>388</v>
-      </c>
-      <c r="E60" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="F60" s="9" t="s">
-        <v>343</v>
-      </c>
-      <c r="G60" t="s">
-        <v>357</v>
-      </c>
-      <c r="J60" s="9" t="s">
-        <v>417</v>
       </c>
       <c r="K60" s="18">
         <v>44865</v>
@@ -3292,10 +3292,10 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D61" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>238</v>
@@ -3330,25 +3330,25 @@
         <v>2</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D63" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>252</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G63" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="H63" t="s">
         <v>285</v>
       </c>
       <c r="J63" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="K63" s="28">
         <v>4000</v>
@@ -3365,25 +3365,25 @@
         <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D64" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E64" s="9" t="s">
         <v>252</v>
       </c>
       <c r="F64" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G64" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="H64" t="s">
         <v>285</v>
       </c>
       <c r="J64" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="K64" s="41">
         <v>50</v>
@@ -3400,25 +3400,25 @@
         <v>2</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D65" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>252</v>
       </c>
       <c r="F65" s="9" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G65" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="H65" t="s">
         <v>285</v>
       </c>
       <c r="J65" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="K65" s="18">
         <v>44925</v>
@@ -3435,28 +3435,28 @@
         <v>1</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D66" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E66" s="9" t="s">
         <v>252</v>
       </c>
       <c r="F66" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="G66" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="H66" t="s">
         <v>285</v>
       </c>
       <c r="J66" t="s">
+        <v>430</v>
+      </c>
+      <c r="K66" s="30" t="s">
         <v>431</v>
-      </c>
-      <c r="K66" s="30" t="s">
-        <v>432</v>
       </c>
       <c r="L66" s="21">
         <v>0.16900000000000001</v>
@@ -3470,10 +3470,10 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D67" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>86</v>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="H67" s="9"/>
       <c r="J67" s="9" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="K67" s="28">
         <v>120000</v>
@@ -3503,23 +3503,23 @@
         <v>1</v>
       </c>
       <c r="C68" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D68" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E68" s="9" t="s">
         <v>86</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="G68" s="9">
         <v>603</v>
       </c>
       <c r="H68" s="9"/>
       <c r="J68" s="9" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="K68" s="28">
         <v>39000</v>
@@ -3536,10 +3536,10 @@
         <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D69" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>86</v>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="H69" s="9"/>
       <c r="J69" s="9" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="K69" s="28">
         <v>180000</v>
@@ -3569,16 +3569,16 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D70" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E70" t="s">
         <v>158</v>
       </c>
       <c r="F70" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="G70" t="s">
         <v>281</v>
@@ -3587,7 +3587,7 @@
         <v>285</v>
       </c>
       <c r="J70" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K70" s="28">
         <v>81000</v>
@@ -3690,7 +3690,7 @@
         <v>205</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E74" s="14" t="s">
         <v>88</v>
@@ -3762,7 +3762,7 @@
         <v>212</v>
       </c>
       <c r="D76" s="14" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E76" s="14" t="s">
         <v>88</v>
@@ -3796,7 +3796,7 @@
         <v>236</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>88</v>
@@ -3815,7 +3815,7 @@
         <v>233</v>
       </c>
       <c r="K77" s="30" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="L77" s="31">
         <v>1.91</v>
@@ -3834,7 +3834,7 @@
         <v>209</v>
       </c>
       <c r="D78" s="14" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E78" s="14" t="s">
         <v>88</v>
@@ -3874,7 +3874,7 @@
         <v>243</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E80" s="9" t="s">
         <v>242</v>
@@ -3883,7 +3883,7 @@
         <v>241</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="I80" s="5"/>
       <c r="J80" s="9" t="s">
@@ -3912,10 +3912,10 @@
         <v>5</v>
       </c>
       <c r="C82" s="42" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D82" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="L82" s="21"/>
       <c r="M82" s="21"/>
@@ -3925,10 +3925,10 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D83" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="L83" s="21"/>
       <c r="M83" s="21"/>
@@ -3938,10 +3938,10 @@
         <v>1</v>
       </c>
       <c r="C84" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="D84" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="L84" s="21"/>
       <c r="M84" s="21"/>
@@ -3954,19 +3954,19 @@
         <v>279</v>
       </c>
       <c r="D85" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E85" t="s">
         <v>277</v>
       </c>
       <c r="F85" t="s">
+        <v>419</v>
+      </c>
+      <c r="G85" t="s">
+        <v>446</v>
+      </c>
+      <c r="J85" t="s">
         <v>420</v>
-      </c>
-      <c r="G85" t="s">
-        <v>447</v>
-      </c>
-      <c r="J85" t="s">
-        <v>421</v>
       </c>
       <c r="K85" s="18">
         <v>44557</v>
@@ -3985,10 +3985,10 @@
         <v>1</v>
       </c>
       <c r="C86" s="42" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D86" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="L86" s="21"/>
       <c r="M86" s="21"/>
@@ -4001,7 +4001,7 @@
         <v>278</v>
       </c>
       <c r="D87" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E87" t="s">
         <v>277</v>
@@ -4010,7 +4010,7 @@
         <v>276</v>
       </c>
       <c r="G87" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="J87" t="s">
         <v>275</v>
@@ -4032,10 +4032,10 @@
         <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D88" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="K88" s="17"/>
       <c r="L88" s="21"/>
@@ -4048,13 +4048,13 @@
         <v>1</v>
       </c>
       <c r="C89" s="42" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D89" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G89" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="L89" s="21"/>
       <c r="M89" s="21"/>

</xml_diff>

<commit_message>
- Steckverbinder Signal und Lock aktualisiert
</commit_message>
<xml_diff>
--- a/BOM/20211102 BOM TeKaDe Baseboard.xlsx
+++ b/BOM/20211102 BOM TeKaDe Baseboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IngBuero\Projekte_Kunden\2021_TeKaDeRevival\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9756184-5EF5-4245-88E4-CD3D31CBEFCF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFADFD3D-C675-46A7-8B4A-71A144231116}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11960" xr2:uid="{261E8F2A-9F01-4E4B-AED6-14B6866C8B8C}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="458">
   <si>
     <t>SOT-23</t>
   </si>
@@ -1372,13 +1372,34 @@
     <t>J11</t>
   </si>
   <si>
-    <t>Pinheader 1x03 P2,54</t>
-  </si>
-  <si>
-    <t>Pinheader 1x02 P2,54</t>
-  </si>
-  <si>
     <t>150R/1%</t>
+  </si>
+  <si>
+    <t>53048-0250</t>
+  </si>
+  <si>
+    <t>Molex</t>
+  </si>
+  <si>
+    <t>PicoBlade</t>
+  </si>
+  <si>
+    <t>538-53048-0250</t>
+  </si>
+  <si>
+    <t>53048-0350</t>
+  </si>
+  <si>
+    <t>538-53048-0350</t>
+  </si>
+  <si>
+    <t>ATMega Pinhead 1x03 P2,54</t>
+  </si>
+  <si>
+    <t>Lock Connector 1x03 P1,25</t>
+  </si>
+  <si>
+    <t>Signal Connector 1x03 P1,25</t>
   </si>
 </sst>
 </file>
@@ -2358,7 +2379,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D21" t="s">
         <v>375</v>
@@ -3925,7 +3946,7 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="D83" t="s">
         <v>398</v>
@@ -3938,13 +3959,32 @@
         <v>1</v>
       </c>
       <c r="C84" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="D84" t="s">
         <v>399</v>
       </c>
-      <c r="L84" s="21"/>
-      <c r="M84" s="21"/>
+      <c r="E84" t="s">
+        <v>450</v>
+      </c>
+      <c r="F84" t="s">
+        <v>449</v>
+      </c>
+      <c r="G84" t="s">
+        <v>451</v>
+      </c>
+      <c r="J84" t="s">
+        <v>452</v>
+      </c>
+      <c r="K84" s="17">
+        <v>3400</v>
+      </c>
+      <c r="L84" s="21">
+        <v>0.503</v>
+      </c>
+      <c r="M84" s="21">
+        <v>0.307</v>
+      </c>
     </row>
     <row r="85" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B85">
@@ -4032,14 +4072,32 @@
         <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="D88" t="s">
         <v>447</v>
       </c>
-      <c r="K88" s="17"/>
-      <c r="L88" s="21"/>
-      <c r="M88" s="21"/>
+      <c r="E88" t="s">
+        <v>450</v>
+      </c>
+      <c r="F88" t="s">
+        <v>453</v>
+      </c>
+      <c r="G88" t="s">
+        <v>451</v>
+      </c>
+      <c r="J88" t="s">
+        <v>454</v>
+      </c>
+      <c r="K88" s="17">
+        <v>12800</v>
+      </c>
+      <c r="L88" s="21">
+        <v>0.59499999999999997</v>
+      </c>
+      <c r="M88" s="21">
+        <v>0.39600000000000002</v>
+      </c>
       <c r="N88" s="21"/>
       <c r="O88" s="21"/>
     </row>

</xml_diff>